<commit_message>
Classify SAMPLE BAG under 8531 90 00 00
The SAMPLE BAG line carries no ONTIME code on either the invoice or the
packing list and is absent from the VTOP HS code key. Confirmed by the
client that it belongs under an existing code; booked to 8531 90 00 00
and merged into that row.

Supporting evidence: 10.50 kg / 1,000 pcs = 10.5 g per piece, matching
the HD hard-tag range (HD2051 = 10.9 g/pc) rather than empty poly bags.

Summary is now 7 rows; totals unchanged and still reconciled to the
invoice and packing list.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019EyVp4rzuRSApof3Yg9s8R
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_V-TOP_EUROPE_WPXA26B0826CZ501.xlsx
+++ b/output/HS_Code_Summary_V-TOP_EUROPE_WPXA26B0826CZ501.xlsx
@@ -44,7 +44,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -58,17 +58,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF6969"/>
+        <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
+        <fgColor rgb="FFFF6969"/>
       </patternFill>
     </fill>
     <fill>
@@ -133,21 +138,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -513,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -611,7 +616,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Části a součásti elektrických signalizačních přístrojů (EAS) – pevné samoobslužné schránky AM či RF (Double, Single, Triple Protection Box Wrap, Alarm Box) s magnetickým zámkem; pevné samoobslužné štítky s magnetickým kabelovým zámkem; štítky AM nebo RF s ocelovým nebo plastovým kabelem k ochraně lahví a plechovek; standardní tvrdé etikety (štítky) k ochraně textilu, oděvů a příslušenství – technologie RF / AM / RF &amp; AM a magnetický zámek. Určeno k ochraně zboží proti krádeži v obchodech.</t>
+          <t>Části a součásti elektrických signalizačních přístrojů (EAS) – pevné samoobslužné schránky AM či RF (Double, Single, Triple Protection Box Wrap, Alarm Box) s magnetickým zámkem; pevné samoobslužné štítky s magnetickým kabelovým zámkem; štítky AM nebo RF s ocelovým nebo plastovým kabelem k ochraně lahví a plechovek; standardní tvrdé etikety (štítky) k ochraně textilu, oděvů a příslušenství – technologie RF / AM / RF &amp; AM a magnetický zámek. Určeno k ochraně zboží proti krádeži v obchodech. Včetně vzorků štítků dodaných ve vzorkovém sáčku (položka SAMPLE BAG).</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -620,19 +625,19 @@
         </is>
       </c>
       <c r="E2" s="3" t="n">
-        <v>259100</v>
+        <v>260100</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>4340.4</v>
+        <v>4350.9</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4665</v>
+        <v>4676.1</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>4794.09</v>
+        <v>4805.5</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>38250.08</v>
+        <v>38270.08</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -641,11 +646,15 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>AS1038, AS1002E, AS1103E, AS1001E, BT3042, BT3055, HD2001, HD2030, HD2051, HD2085, HD2150, HD2045, HD2036, BT3018</t>
+          <t>AS1038, AS1002E, AS1103E, AS1001E, BT3042, BT3055, HD2001, HD2030, HD2051, HD2085, HD2150, HD2045, HD2036, BT3018, SAMPLE BAG</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>Zahrnuje položku SAMPLE BAG (1 000 ks, 10,5 g/ks, 20,00 EUR) – na faktuře i packing listu bez kódu ONTIME. Zařazena k tomuto kódu na základě potvrzení klienta; hmotnost na kus odpovídá tvrdým štítkům řady HD.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="58" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -702,7 +711,7 @@
           <t>HANGZHOU ONTIME I.T. CO., LTD., Hangzhou, CHINA</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>8205 59 80 00</t>
         </is>
@@ -742,12 +751,12 @@
           <t>DL4405 KEY, DT4002</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="6" t="inlineStr">
         <is>
           <t>POZOR – KÓD ZMĚNĚN</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>V klíči byl u DL4405 KEY kód 7326 90 98 90 PŘEŠKRTNUT (neplatný) – použit platný kód 8205 59 80 00. Pozn.: 7326 je zboží CBAM, 8205 nikoli.</t>
         </is>
@@ -954,217 +963,160 @@
       <c r="M8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>HANGZHOU ONTIME I.T. CO., LTD., Hangzhou, CHINA</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>NEZAŘAZENO</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>SAMPLE BAG (vzorkový sáček) – položka není uvedena v sazebníkovém klíči VTOP EUROPE (HS kódy 10.9.2026). HS kód nutno doplnit před podáním CP.</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>11.41</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>CFR Praha (CFR PRAGUE)</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>SAMPLE BAG</t>
-        </is>
-      </c>
-      <c r="L9" s="6" t="inlineStr">
-        <is>
-          <t>CHYBÍ HS KÓD</t>
-        </is>
-      </c>
-      <c r="M9" s="6" t="inlineStr">
-        <is>
-          <t>CHYBÍ HS KÓD – položka SAMPLE BAG není v sazebníkovém klíči. Nutno doplnit před podáním CP.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr"/>
-      <c r="C10" s="7" t="inlineStr"/>
-      <c r="D10" s="7" t="inlineStr"/>
-      <c r="E10" s="8" t="n">
+      <c r="B9" s="7" t="inlineStr"/>
+      <c r="C9" s="7" t="inlineStr"/>
+      <c r="D9" s="7" t="inlineStr"/>
+      <c r="E9" s="8" t="n">
         <v>500554</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F9" s="9" t="n">
         <v>4536</v>
       </c>
-      <c r="G10" s="9" t="n">
+      <c r="G9" s="9" t="n">
         <v>4878</v>
       </c>
-      <c r="H10" s="9" t="n">
+      <c r="H9" s="9" t="n">
         <v>5013</v>
       </c>
-      <c r="I10" s="9" t="n">
+      <c r="I9" s="9" t="n">
         <v>43377.18</v>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="J9" s="7" t="inlineStr">
         <is>
           <t>CFR Praha</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr"/>
-      <c r="L10" s="7" t="inlineStr"/>
-      <c r="M10" s="7" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>LEGENDA A KONTROLNÍ SOUČTY</t>
         </is>
       </c>
     </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>🔵 MODRÁ</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Položka bez kódu ONTIME na faktuře – zařazena na základě potvrzení klienta, viz poznámka u kódu 8531 90 00 00.</t>
+        </is>
+      </c>
+    </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>🔴 ČERVENÁ</t>
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>🟠 ORANŽOVÁ</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Chybějící HS kód – nutno doplnit před podáním celního prohlášení.</t>
+          <t>HS kód v sazebníkovém klíči přeškrtnut / nahrazen – ověřeno a použit platný kód.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>🟠 ORANŽOVÁ</t>
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Zásilka</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>HS kód v sazebníkovém klíči přeškrtnut / nahrazen – ověřeno a použit platný kód.</t>
+          <t>Odesílatel: HANGZHOU ONTIME I.T. CO., LTD., Hangzhou, Čína  |  Příjemce: V-TOP EUROPE s.r.o., Františka Diviše 1012/64, 104 00 Praha 22 Uhříněves, IČO 257 95 040, DIČ CZ25795040</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>Zásilka</t>
+          <t>Doklady</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Odesílatel: HANGZHOU ONTIME I.T. CO., LTD., Hangzhou, Čína  |  Příjemce: V-TOP EUROPE s.r.o., Františka Diviše 1012/64, 104 00 Praha 22 Uhříněves, IČO 257 95 040, DIČ CZ25795040</t>
+          <t>Faktura PI24200070026048B&amp;053&amp;054B ze dne 14.8.2026; Packing list k téže faktuře; potvrzení přepravy WPXA26B0826CZ501 (železniční přeprava Xi'an → Khorgos → Praha, odjezd 2.9.2026, 40HC NWRU8624306/003451032, CFS-CFS, freight prepaid).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>Doklady</t>
+          <t>Incoterms</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Faktura PI24200070026048B&amp;053&amp;054B ze dne 14.8.2026; Packing list k téže faktuře; potvrzení přepravy WPXA26B0826CZ501 (železniční přeprava Xi'an → Khorgos → Praha, odjezd 2.9.2026, 40HC NWRU8624306/003451032, CFS-CFS, freight prepaid).</t>
+          <t>CFR PRAGUE (CFR Praha) – uvedeno v poli TERMS obchodní faktury. Přepravné do Prahy je součástí fakturované ceny. Pozn.: CFR je doložka určená pro námořní/vnitrozemskou vodní přepravu, zde použita pro železniční přepravu – doporučeno ověřit s klientem (věcně odpovídá CPT Praha).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>Incoterms</t>
+          <t>Množství</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>CFR PRAGUE (CFR Praha) – uvedeno v poli TERMS obchodní faktury. Přepravné do Prahy je součástí fakturované ceny. Pozn.: CFR je doložka určená pro námořní/vnitrozemskou vodní přepravu, zde použita pro železniční přepravu – doporučeno ověřit s klientem (věcně odpovídá CPT Praha).</t>
+          <t>500 554 ks – souhlasí s fakturou i packing listem.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>Množství</t>
+          <t>Hmotnosti</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>500 554 ks – souhlasí s fakturou i packing listem.</t>
+          <t>Čistá 4 536,00 kg; hrubá dle položek 4 878,00 kg; palety (9 ks) 135,00 kg; hrubá celkem 5 013,00 kg. Sloupec „Hrubá hmotnost vč. palet“ rozpouští tāru palet poměrně dle hrubé hmotnosti položek (faktor 1,027675).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>Hmotnosti</t>
+          <t>Celní hodnota</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Čistá 4 536,00 kg; hrubá dle položek 4 878,00 kg; palety (9 ks) 135,00 kg; hrubá celkem 5 013,00 kg. Sloupec „Hrubá hmotnost vč. palet“ rozpouští tāru palet poměrně dle hrubé hmotnosti položek (faktor 1,027675).</t>
+          <t>43 377,18 EUR – souhlasí se součtem faktury (SUB TOTAL = TOTAL). Obchodní sleva nebyla na faktuře uplatněna, proporcionální rozpočet slevy se proto neprovádí.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Celní hodnota</t>
+          <t>Sloučení</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>43 377,18 EUR – souhlasí se součtem faktury (SUB TOTAL = TOTAL). Obchodní sleva nebyla na faktuře uplatněna, proporcionální rozpočet slevy se proto neprovádí.</t>
+          <t>Řádky faktury sloučeny na unikátní HS kódy v rámci jednoho odesílatele (32 řádků faktury → 7 řádků). Zásilka má jediného odesílatele, proto nedochází ke kolizi stejného HS kódu napříč odesílateli.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>Sloučení</t>
+          <t>Zdroj popisů</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>Řádky faktury sloučeny na unikátní HS kódy v rámci jednoho odesílatele (32 řádků faktury → 8 řádků). Zásilka má jediného odesílatele, proto nedochází ke kolizi stejného HS kódu napříč odesílateli.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>Zdroj popisů</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
         <is>
           <t>Sazebníkový klíč „VTOP EUROPE s.r.o. – HS kódy 10.9.2026.xlsx“, list List1. U kódů 3926 90 97 90 a 8205 59 80 00 použit „Návrh popisu do CP“. Text popisu u 3926 90 97 90 je ve zdrojovém souboru useknutý („…proti použit“) – doplněno na „proti neoprávněnému použití“, doporučeno potvrdit.</t>
         </is>
@@ -1173,8 +1125,8 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="C20:M20"/>
+    <mergeCell ref="C12:M12"/>
     <mergeCell ref="C21:M21"/>
-    <mergeCell ref="C22:M22"/>
     <mergeCell ref="C15:M15"/>
     <mergeCell ref="C16:M16"/>
     <mergeCell ref="C19:M19"/>
@@ -1501,22 +1453,22 @@
       <c r="B29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>OTEVŘENÉ BODY K DOŘEŠENÍ</t>
         </is>
       </c>
-      <c r="B30" s="16" t="inlineStr"/>
+      <c r="B30" s="19" t="inlineStr"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>1) SAMPLE BAG</t>
+          <t>1) SAMPLE BAG – VYŘEŠENO</t>
         </is>
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>1 000 ks / 10,50 kg net / 20,00 EUR – chybí HS kód v sazebníkovém klíči. Nutno doplnit před podáním CP.</t>
+          <t>1 000 ks / 10,50 kg net / 20,00 EUR. Na faktuře ani na packing listu není uveden kód ONTIME a položka není v sazebníkovém klíči. Po potvrzení klientem zařazena pod 8531 90 00 00 (vzorky štítků) a sloučena do tohoto řádku. Podpůrný argument: 10,50 kg / 1 000 ks = 10,5 g na kus, což odpovídá tvrdým štítkům řady HD (HD2051 = 10,9 g/ks), nikoli prázdným plastovým sáčkům (jinak 3923 21 00 00).</t>
         </is>
       </c>
     </row>

</xml_diff>